<commit_message>
se parametriza la creacion de carpetas de albumes y artistas automaticamente
</commit_message>
<xml_diff>
--- a/music.xlsx
+++ b/music.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PYTHON\music_download\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF48B923-1156-4493-9E3F-586D84576A29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEAE7EE3-0F2D-41B1-90C6-8DA0EA40DF0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="PXNDX" sheetId="2" r:id="rId2"/>
-    <sheet name="GUNS N' ROSES" sheetId="3" r:id="rId3"/>
+    <sheet name="PXNDX" sheetId="2" r:id="rId1"/>
+    <sheet name="Guns N' Roses" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,64 +26,63 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
-  <si>
-    <t>PXNDX</t>
-  </si>
-  <si>
-    <t>GUNS N' ROSES</t>
-  </si>
-  <si>
-    <t>LINKIN PARK</t>
-  </si>
-  <si>
-    <t>Amantes Sunt Amentes</t>
-  </si>
-  <si>
-    <t>La Estrategia Perdida</t>
-  </si>
-  <si>
-    <t>So Violento So Macabro</t>
-  </si>
-  <si>
-    <t>Para Ti Con Desprecio</t>
-  </si>
-  <si>
-    <t>Reflexiones de una Mente Perturbada</t>
-  </si>
-  <si>
-    <t>Disculpa los Malos Pensamientos</t>
-  </si>
-  <si>
-    <t>Poetics</t>
-  </si>
-  <si>
-    <t>Bonanza</t>
-  </si>
-  <si>
-    <t>Sangre Fría</t>
-  </si>
-  <si>
-    <t>Sinfonia Soledad</t>
-  </si>
-  <si>
-    <t>APTETITO DE DESTRUCCION</t>
-  </si>
-  <si>
-    <t>YO COULD BE MINE</t>
-  </si>
-  <si>
-    <t>DON'T CRY</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_nhExNbsuT4shEKEVHqc_8VCjpfjJFT_lc</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_loKqS03yOG47kKz8c6t_TQDvKtwFVCcwc</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_lD32fKOjxVNwRN8aFrLvi3Gs7Kw781mks</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_mgLfmjWSBBRCZw8-7uPQncbKG7P9jdQHc</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_kk8_zS51PxQKlUMAMn8ERMdvnsV4YuvFA</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_mMIbVwHJnElfLj_MJ65vKf5sO81uyl0Qo</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_nrZfcw3kEy3JROCsg7cBfetVazE94Nxp0</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_mqTL3PIyxGBNNWg8fdb86PJBtoPJwdPNU</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_lBFwKbOYWuj1MjWRuUGTiVc1Y58Jaa8Sw</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_meSzJKrAICsYqnF4wrZZbywJ19Qkexi7A</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_ltQiuNnoBifeiEYSjm5Ac1Z-x3ydiYrq4</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_niWwBZzVmo7rEL2WwKOIArwgbBmLBjB64</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_llbiwWjwlRC6554PAK85FIRT10WsgIWlY</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -107,16 +105,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -394,79 +393,55 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74637DD3-FA64-4A0E-907E-B7E37CFE0BF0}">
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="26.77734375" customWidth="1"/>
-    <col min="3" max="3" width="25.5546875" customWidth="1"/>
+    <col min="1" max="1" width="76.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="76.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="78.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="74.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="78.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="76.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="75.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="78.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="75.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
-        <v>1</v>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74637DD3-FA64-4A0E-907E-B7E37CFE0BF0}">
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="24" style="1" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" style="1" customWidth="1"/>
-    <col min="3" max="4" width="8.88671875" style="1"/>
-    <col min="5" max="5" width="12.109375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="16.109375" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.88671875" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>8</v>
-      </c>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -474,25 +449,26 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F7FBE45-576C-4B74-858E-A0B1ACAB2C58}">
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF96CC9E-6A2D-40A9-820D-A4D962E5B60F}">
   <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.21875" customWidth="1"/>
-    <col min="2" max="2" width="23.21875" customWidth="1"/>
-    <col min="3" max="3" width="16.33203125" customWidth="1"/>
+    <col min="1" max="1" width="73.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="79.21875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="75.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C1" t="s">
-        <v>15</v>
+      <c r="A1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ultima actualizacion antes de pasar a linux, toca arreglar todo lo de las ruta de los archivos
</commit_message>
<xml_diff>
--- a/music.xlsx
+++ b/music.xlsx
@@ -1,20 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PYTHON\music_download\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEAE7EE3-0F2D-41B1-90C6-8DA0EA40DF0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4030BEE6-5271-4431-AA87-034138C2DFF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PXNDX" sheetId="2" r:id="rId1"/>
     <sheet name="Guns N' Roses" sheetId="3" r:id="rId2"/>
+    <sheet name="Linkin Park" sheetId="4" r:id="rId3"/>
+    <sheet name="Red Hot Chili Peppers" sheetId="5" r:id="rId4"/>
+    <sheet name="Paramore" sheetId="6" r:id="rId5"/>
+    <sheet name="Green Day" sheetId="7" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="58">
   <si>
     <t>https://music.youtube.com/playlist?list=OLAK5uy_nhExNbsuT4shEKEVHqc_8VCjpfjJFT_lc</t>
   </si>
@@ -65,6 +69,141 @@
   </si>
   <si>
     <t>https://music.youtube.com/playlist?list=OLAK5uy_llbiwWjwlRC6554PAK85FIRT10WsgIWlY</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_mSTK5j-BifeC6mHoSjMC5qI-U0MgDoNHU</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_lwKwguxJSAvoH4l1fruQIIJjp4Eeod37U</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_lGBK0LgMwE5DbbS6r3U31rUzfU9IZrFtw</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_nGSVnT8Dd85NFcqrFWHGbEBzgKT6uV6m0</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_mc5PauMftpwP2SEGmQEb1V9146Q9hT18A</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_l7Hs3PJjpSoB0r91uBoUGqbtSulyXeIAA</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_kHLHm6L9JGlCys4egnA8x8ZDpMx0dMwBQ</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_kIzyG7Jg7kBISY4qgyTJRPr2pUGH4f9nY</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_kCKoxuwJvJeFIAAMTkgHOaZHP64m0fZPg</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_mfCBTt0IqG8aeK8iTJuwIbnm6W8fpB49Q</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_mMmS4TSrWwYr9qs5g4QQ1U8rFIDEdKIhY</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_ncbxWnjKunOOgJ7N1XELrneNgiaMMPXxA</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_nIS-c5OD2p7LJU3n8S_tcu6q2QzBe-vzM</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_krvx3FeVGumNUfYCsbaL0ikF--a7KJ55U</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_lfNmExJs6xV-8ApZL4zicCfFVzfv-w8cI</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_kDBTPFjTRerD0gAG3g4Xs3UxGQSzZBoZQ</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_lzoqSoDPX9PH9TC6_jUP3URbLJdQXzRPo</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_lL9dW1Y3Mm0MHkCrvhc12h1J3Qqrzj7-I</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_kwp9Hk00Ynjv-z4eYlhEA1nVdqL51Y2ac</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_kTnNQq084U1cNShZyo2NpbMRg2-bbuMco</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_mMa5i7OJDtHbIxX8Vl87xVzphCfy24Bhw</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_nkWxw1Aw8K8Qt7-wX9Z-L_vw0vwKpK2s4</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_mSdHwQhtcUy4eD_I_d4ppchtxeHXBgZA8</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_mNXrSc9X8kS3dRXOSxcMY3f-wrVboj0wM</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_mPLwBYr_pP0i7gg3Kq2WNykTfNGN5TXLQ</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_nqzWv4aFRNiymgpQ6uFhYya3TwLh1ksHg</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_kLAfOEEj-Z_CPY9xPP-n55QhP41qlv7nY</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_k0ji2bfpRw9H7luk2AajXQP8dR-oVK97k</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_mkmsiYxs2e_K4ppqU5IDUslZbb_wQEQ1o</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_ma8O0EMQh5gIfu0LWSW7dQAUnzEb8NVIU</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_msBP0AmgnhfaownQDTYhhzdjWnnlgRNOc</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_l-Rd8aIoTqerGzAYt2UBWCA9lmNY_slEw</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_k3wiQCUAyNFLiMpLR-lA7rDnBUfJFXsWI</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_kejZkcg7neNpxst8p72bcTYnsgo1a9ofY</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_mrF_EHJJul_9cUfE-snfFgdEY_nggl9c0</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_nALXtvN4rRXq8IpDbSSlYTuTcO4L4YBGE</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_mmM6IEvxyWMmJhYOVc3YyFUH7espfFHP4</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_mIFn-YhTNCRYPqK2czZKEakLy5Gs6G89Q</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_np1hyyFM8ZG6foL_5lRlhR5B8d-p0Y18c</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_mJteDTUAbcYY1YzRfoDaXCKzzPZ8NzTng</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_n0piktiaFmxEHhytR_fPmVfxmT-jj2bB0</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_mhM9Ks_S0deTeTD7UqpoHx1F-3YAuLQ-0</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_mc9Z_uiv7QlX3I3Rn72KUu77W2A6foMCA</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_nmMRcBPEXxsWW5l7T5kYIDH8WG5Hrd1v0</t>
+  </si>
+  <si>
+    <t>https://music.youtube.com/playlist?list=OLAK5uy_n4q5YXrgrCOE_aKIU94xFaK4_gUyQXOwM</t>
   </si>
 </sst>
 </file>
@@ -112,7 +251,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -451,27 +590,277 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF96CC9E-6A2D-40A9-820D-A4D962E5B60F}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:Q1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="73.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="79.21875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="75.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="8.88671875" style="2"/>
+    <col min="1" max="1" width="73.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="79.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="75.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="78.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="74.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="76.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="78.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="79.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="74.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="74.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="78.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="77.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="78.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" t="s">
         <v>12</v>
+      </c>
+      <c r="D1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E1" r:id="rId1" xr:uid="{A6B1C19C-A659-4BC8-8A18-4BC33F0E5C6F}"/>
+    <hyperlink ref="G1" r:id="rId2" xr:uid="{FADE3C88-CBD9-4A97-82AE-9C78A2CBF67C}"/>
+    <hyperlink ref="H1" r:id="rId3" xr:uid="{7FF31555-C949-4402-B6B6-725630DBF4A6}"/>
+    <hyperlink ref="I1" r:id="rId4" xr:uid="{7246E1B5-6BF8-44AC-9960-B19629FC3D7A}"/>
+    <hyperlink ref="K1" r:id="rId5" xr:uid="{C44B7864-54A4-46C7-904D-373298D35F65}"/>
+    <hyperlink ref="J1" r:id="rId6" xr:uid="{7AABB435-EE42-4606-BB1B-9F18995C765E}"/>
+    <hyperlink ref="L1" r:id="rId7" xr:uid="{55ECB4FC-5C2F-4AAA-9856-D7A297F592A4}"/>
+    <hyperlink ref="M1" r:id="rId8" xr:uid="{2D8D76AD-E983-4CDB-A1A8-DB3DFB150EDD}"/>
+    <hyperlink ref="F1" r:id="rId9" xr:uid="{62E64958-B552-4330-B83E-FD7F01C0109B}"/>
+    <hyperlink ref="N1" r:id="rId10" xr:uid="{059723E7-B469-4B19-BABD-AB3911506D54}"/>
+    <hyperlink ref="O1" r:id="rId11" xr:uid="{09FF2F90-AA69-42CB-A522-4AC34C09E711}"/>
+    <hyperlink ref="Q1" r:id="rId12" xr:uid="{EEC451D2-DC7A-4BB0-92B7-3BF207C10AAE}"/>
+    <hyperlink ref="P1" r:id="rId13" xr:uid="{464F924F-F32E-467F-9D77-12B7D085D664}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC51DA85-8D64-4A85-844E-C5839E4CB742}">
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="2" width="77.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="75.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="73.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="77.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="76.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="76.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B1" r:id="rId1" xr:uid="{BAD97AF6-2D48-404E-9773-C45ADEF07445}"/>
+    <hyperlink ref="A1" r:id="rId2" xr:uid="{EF20BAC7-D535-4314-9603-A1661D2C15A3}"/>
+    <hyperlink ref="C1" r:id="rId3" xr:uid="{6D8683F4-A66E-46CF-90B5-4754F4881671}"/>
+    <hyperlink ref="D1" r:id="rId4" xr:uid="{927DA7FB-F904-43A6-9CDB-675E9EB0B39B}"/>
+    <hyperlink ref="E1" r:id="rId5" xr:uid="{6ED781A0-FCB3-495A-9813-C043A3BD729B}"/>
+    <hyperlink ref="F1" r:id="rId6" xr:uid="{013E8939-DF97-4006-8E46-EA86D4B05732}"/>
+    <hyperlink ref="G1" r:id="rId7" xr:uid="{D91EDB2D-233D-4B7F-ABA3-2203F9AC3365}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F41BF2D-B17B-4304-8A69-96AA3BCEC09C}">
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" r:id="rId1" xr:uid="{C296C337-1B00-4802-96A0-4390C4244F86}"/>
+    <hyperlink ref="B1" r:id="rId2" xr:uid="{3A835BCE-8D0C-4F73-ADCD-527F7E5A0170}"/>
+    <hyperlink ref="C1" r:id="rId3" xr:uid="{E12877E0-53D3-44A1-A584-08F734860C5E}"/>
+    <hyperlink ref="D1" r:id="rId4" xr:uid="{F68AB639-1DC6-474A-B536-F149BFEB834E}"/>
+    <hyperlink ref="E1" r:id="rId5" xr:uid="{30C914DE-6FD9-4E3F-A2D5-AF483D90F41F}"/>
+    <hyperlink ref="F1" r:id="rId6" xr:uid="{79B44C57-039A-4AE7-B224-7CA0D1C86966}"/>
+    <hyperlink ref="G1" r:id="rId7" xr:uid="{8D9C7DF7-2ABE-4A11-897C-672669CB3319}"/>
+    <hyperlink ref="H1" r:id="rId8" xr:uid="{023F06C1-F399-4AB9-AE0D-7735271B66E1}"/>
+    <hyperlink ref="I1" r:id="rId9" xr:uid="{0CB70635-DD36-40EC-BF01-F089B2C92548}"/>
+    <hyperlink ref="K1" r:id="rId10" xr:uid="{304096D1-7827-4C5D-B29A-8CA247D0F5D4}"/>
+    <hyperlink ref="J1" r:id="rId11" xr:uid="{E9F52E38-645C-4012-9956-B71CAF7BB053}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78AC2578-D409-4B33-8956-5DDB6C142200}">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" r:id="rId1" xr:uid="{7ED6FFBA-76D2-4C66-BF8E-93A5E0373CA7}"/>
+    <hyperlink ref="B1" r:id="rId2" xr:uid="{81A91D7D-10A0-4376-9BF8-D2D3A7C0C0FA}"/>
+    <hyperlink ref="C1" r:id="rId3" xr:uid="{F25BFF31-CD25-479C-A480-416B6A5D762E}"/>
+    <hyperlink ref="D1" r:id="rId4" xr:uid="{AD74674D-88E3-4368-818C-A488DFD24E10}"/>
+    <hyperlink ref="E1" r:id="rId5" xr:uid="{49F44BC6-C2CE-42F0-AB8E-70BC124D8EA9}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC2D9AC0-0730-462C-849A-8800D2D7F673}">
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G1" t="s">
+        <v>53</v>
+      </c>
+      <c r="H1" t="s">
+        <v>54</v>
+      </c>
+      <c r="I1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B1" r:id="rId1" xr:uid="{08207C0D-D96F-4FCA-B4E3-01A504002AB7}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>